<commit_message>
Person Excel Export, その他、ほぼ完成
</commit_message>
<xml_diff>
--- a/models/data/field.xlsx
+++ b/models/data/field.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D31F8667-4087-4795-812F-D7FB8AC4D77F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E2570DD-3201-42E7-A8D3-0CCF592BA086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5400" yWindow="1995" windowWidth="22695" windowHeight="13065" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="22695" windowHeight="13065" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="岩座神農地" sheetId="1" r:id="rId1"/>
@@ -182,7 +182,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -242,25 +242,25 @@
     <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="179" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="176" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="177" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -580,40 +580,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="17" t="s">
         <v>6</v>
       </c>
     </row>
@@ -635,16 +635,16 @@
       <c r="I2" s="8"/>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
-      <c r="L2" s="16"/>
+      <c r="L2" s="13"/>
     </row>
     <row r="3" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D3" s="14"/>
-      <c r="E3" s="15">
+      <c r="D3" s="11"/>
+      <c r="E3" s="12">
         <f>D3/100</f>
         <v>0</v>
       </c>
-      <c r="F3" s="14"/>
-      <c r="G3" s="15">
+      <c r="F3" s="11"/>
+      <c r="G3" s="12">
         <f>F3/100</f>
         <v>0</v>
       </c>

</xml_diff>